<commit_message>
Update related scripts and resources
</commit_message>
<xml_diff>
--- a/UI_DESC.xlsx
+++ b/UI_DESC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\worni\Desktop\Ai_GDD\RAID_GDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D8D566-ADC1-4C42-9B34-5594435CDB62}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF45B94-5F42-4825-9715-5CEE6FA8DD56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11175" activeTab="7" xr2:uid="{0B8AA14C-BC36-4293-85B1-BE83A3EAB580}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11175" activeTab="8" xr2:uid="{0B8AA14C-BC36-4293-85B1-BE83A3EAB580}"/>
   </bookViews>
   <sheets>
     <sheet name="parts_pickup_UI_DESC" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="enforce_result_UI" sheetId="6" r:id="rId6"/>
     <sheet name="inven_parts_UI" sheetId="8" r:id="rId7"/>
     <sheet name="inven_parts_change_UI" sheetId="9" r:id="rId8"/>
+    <sheet name="pickup_results_UI" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="89">
   <si>
     <t>번호</t>
   </si>
@@ -580,6 +581,49 @@
     &gt; 테두리 두께: 2px
 - 인벤토리 정렬 우선순위
     &gt; 장착 중인 파츠 → 등급</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1회 뽑기 결과창</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10회 뽑기 결과창</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 뽑기 또는 보상 획득 시 결과 파츠를 중앙에 출력합니다.
+    &gt; 파츠 아이콘 표시
+    &gt; 파츠 이름 표시
+    &gt; 파츠 등급 색상 적용
+    &gt; 예시: 전설 등급 → 노란색
+- 파츠 획득 시 등급에 따른 연출을 출력합니다.
+    &gt; 희귀도별 이펙트 출력 가능
+    &gt; 등장 애니메이션 재생 가능
+- 획득한 파츠를 중앙 강조 형태로 출력합니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 다중 뽑기 시 획득한 파츠 목록을 출력
+    &gt; 그리드 형태 출력
+    &gt; 최대 10개 결과 표시
+- 각 파츠의 정보를 함께 출력
+    &gt; 파츠 아이콘
+    &gt; 파츠 이름
+    &gt; 등급 색상
+- 파츠 등급에 따라 배경 색상을 구분
+    &gt; 파츠 아이콘 표시
+    &gt; 파츠 이름 표시
+    &gt; 파츠 등급 색상 적용
+    &gt; 예시: 전설 등급 → 노란색
+- 획득 순서 기준으로 출력
+    &gt; 좌 → 우
+    &gt; 상 → 하</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 획득 결과 화면을 종료합니다.
+    &gt; 버튼 선택 시 결과창 종료 진행</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -765,6 +809,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -776,9 +823,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1110,7 +1154,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1118,13 +1162,13 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1132,13 +1176,13 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="255" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1146,13 +1190,13 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1160,13 +1204,13 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="183.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1174,13 +1218,13 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="132" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+      <c r="A12" s="9">
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1188,13 +1232,13 @@
       </c>
     </row>
     <row r="13" spans="1:2" ht="191.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
+      <c r="A13" s="9"/>
       <c r="B13" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
+      <c r="A14" s="7">
         <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1202,13 +1246,13 @@
       </c>
     </row>
     <row r="15" spans="1:2" ht="69" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="A15" s="8"/>
       <c r="B15" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
+      <c r="A16" s="9">
         <v>8</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1216,13 +1260,13 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
+      <c r="A17" s="9"/>
       <c r="B17" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="6">
+      <c r="A18" s="7">
         <v>9</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1230,13 +1274,13 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="8"/>
       <c r="B19" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="8">
+      <c r="A20" s="9">
         <v>10</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1244,13 +1288,13 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="8"/>
+      <c r="A21" s="9"/>
       <c r="B21" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
+      <c r="A22" s="7">
         <v>11</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -1258,13 +1302,13 @@
       </c>
     </row>
     <row r="23" spans="1:2" ht="198" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7"/>
+      <c r="A23" s="8"/>
       <c r="B23" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A24" s="8">
+      <c r="A24" s="9">
         <v>12</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1272,13 +1316,13 @@
       </c>
     </row>
     <row r="25" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
+      <c r="A25" s="9"/>
       <c r="B25" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A26" s="6">
+      <c r="A26" s="7">
         <v>13</v>
       </c>
       <c r="B26" s="3" t="s">
@@ -1286,13 +1330,13 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
+      <c r="A27" s="8"/>
       <c r="B27" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="8">
+      <c r="A28" s="9">
         <v>14</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -1300,7 +1344,7 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="173.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="8"/>
+      <c r="A29" s="9"/>
       <c r="B29" s="4" t="s">
         <v>20</v>
       </c>
@@ -1346,7 +1390,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1354,13 +1398,13 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1368,13 +1412,13 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1382,13 +1426,13 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="172.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1396,13 +1440,13 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1410,7 +1454,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>39</v>
       </c>
@@ -1446,7 +1490,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1454,13 +1498,13 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1468,13 +1512,13 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1482,13 +1526,13 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="168.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1496,13 +1540,13 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1510,7 +1554,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="112.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>43</v>
       </c>
@@ -1547,7 +1591,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1555,13 +1599,13 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="131.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1569,13 +1613,13 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="93.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1583,13 +1627,13 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="300" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1597,13 +1641,13 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1611,13 +1655,13 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="150" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
+      <c r="A12" s="7">
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1625,7 +1669,7 @@
       </c>
     </row>
     <row r="13" spans="1:2" ht="150" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
+      <c r="A13" s="10"/>
       <c r="B13" s="4" t="s">
         <v>52</v>
       </c>
@@ -1663,7 +1707,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1671,13 +1715,13 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1685,13 +1729,13 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="225" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1699,21 +1743,21 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="168.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="168.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+    <row r="9" spans="1:2" ht="150" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
       <c r="B9" s="4" t="s">
         <v>52</v>
       </c>
@@ -1749,7 +1793,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1757,13 +1801,13 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="75" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1771,61 +1815,61 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="75" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" spans="1:10" ht="150" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1857,7 +1901,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1865,13 +1909,13 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -1879,94 +1923,94 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="131.25" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" spans="1:10" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
+      <c r="A8" s="7">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" spans="1:10" ht="262.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
+      <c r="A9" s="10"/>
       <c r="B9" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" spans="1:10" ht="131.25" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
     </row>
     <row r="12" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
+      <c r="A12" s="7">
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10" ht="131.25" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
+      <c r="A13" s="10"/>
       <c r="B13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
+      <c r="A14" s="7">
         <v>7</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1974,7 +2018,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
+      <c r="A15" s="10"/>
       <c r="B15" s="4" t="s">
         <v>74</v>
       </c>
@@ -2013,7 +2057,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2021,13 +2065,13 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="75" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="4" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -2035,71 +2079,71 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="112.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" spans="1:10" ht="281.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
+      <c r="A8" s="7">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
+      <c r="A9" s="10"/>
       <c r="B9" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" spans="1:10" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2112,4 +2156,75 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CCE481D-238B-406F-887C-A48BB8BFDB34}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="9"/>
+      <c r="B3" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="10"/>
+      <c r="B5" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="337.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="10"/>
+      <c r="B7" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>